<commit_message>
Added link to slides.
</commit_message>
<xml_diff>
--- a/Schedule.xlsx
+++ b/Schedule.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10201"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10302"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jasonbryer/Dropbox (Personal)/School/Teaching/DAV5300 2026 Spring/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65F0C993-17CE-3641-85EC-45A73CC67FEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFE0192D-3EDE-BF42-B04A-C7D1ECA7577B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1480" yWindow="4680" windowWidth="25340" windowHeight="14540" xr2:uid="{A772458D-4E7B-8249-8B6B-34FE7D5BD316}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="57">
   <si>
     <t>Date</t>
   </si>
@@ -199,6 +199,12 @@
   </si>
   <si>
     <t>/slides/05-Foundation_for_Inference.html</t>
+  </si>
+  <si>
+    <t>/slides/06-Inference_for_Categorical_Data.html</t>
+  </si>
+  <si>
+    <t>/slides/07-Inference_for_Numerical_Data.html</t>
   </si>
 </sst>
 </file>
@@ -701,6 +707,9 @@
       <c r="C7" t="s">
         <v>12</v>
       </c>
+      <c r="D7" t="s">
+        <v>55</v>
+      </c>
       <c r="E7" t="s">
         <v>30</v>
       </c>
@@ -727,6 +736,9 @@
       </c>
       <c r="C9" t="s">
         <v>13</v>
+      </c>
+      <c r="D9" t="s">
+        <v>56</v>
       </c>
       <c r="E9" t="s">
         <v>32</v>

</xml_diff>